<commit_message>
Added debugging code and fixed dialogue
</commit_message>
<xml_diff>
--- a/Noir Wingman/Assets/Sheets/Demo Dialogue/Daria Scarletta/Daria Scarletta 1.0.xlsx
+++ b/Noir Wingman/Assets/Sheets/Demo Dialogue/Daria Scarletta/Daria Scarletta 1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b685ca5cabcdd482/Desktop/NoirWingman/Noir Wingman/Assets/Sheets/Demo Dialogue/Daria Scarletta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="124" documentId="8_{DBC36C78-D6B6-4FCA-A54B-1A49A9FC3B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{391BBD1B-4EC6-4EAC-9B5C-343923FB5964}"/>
+  <xr:revisionPtr revIDLastSave="177" documentId="8_{DBC36C78-D6B6-4FCA-A54B-1A49A9FC3B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6FE2D5A-100C-45C0-8606-AFD61CDCE670}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{4FA77428-4DF4-4557-975A-1859CFCBCEF0}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="76">
   <si>
     <t>Name</t>
   </si>
@@ -89,9 +89,6 @@
     <t>What brings you to the bar tonight?</t>
   </si>
   <si>
-    <t>Null</t>
-  </si>
-  <si>
     <t>3|3</t>
   </si>
   <si>
@@ -155,18 +152,6 @@
     <t xml:space="preserve">*Her eyes narrow for a moment, some kind of mask slipping as she glares at me from over her cocktail, a cruelty you don't often see in 'secretaries'|... |.  .  .|.    .     .|I- uh, I'm sorry.|Mhm  </t>
   </si>
   <si>
-    <t>Angry|Neutral||Angry|Neutral|Angry|Neutral|Neutral|Angry</t>
-  </si>
-  <si>
-    <t>3|0|3|0|3|0|0|3</t>
-  </si>
-  <si>
-    <t>Daria Scarletta|Detective Juels|Daria Scarletta|Detective Juels|Daria Scarletta|Detective Juels|Detective Juels|Daria Scarletta</t>
-  </si>
-  <si>
-    <t>Age</t>
-  </si>
-  <si>
     <t>Add|Add</t>
   </si>
   <si>
@@ -237,6 +222,51 @@
   </si>
   <si>
     <t>Daria Scarletta|Daria Scarletta|Detective Juels|Daria Scarletta|Detective Juels</t>
+  </si>
+  <si>
+    <t>You're deflecting Mrs.Scarletta, hesitant to speak on past relations? (Push it)</t>
+  </si>
+  <si>
+    <t>Relationships 2</t>
+  </si>
+  <si>
+    <t>Resent</t>
+  </si>
+  <si>
+    <t>Subtract</t>
+  </si>
+  <si>
+    <t>Alone|Resent</t>
+  </si>
+  <si>
+    <t>Egt|Egt</t>
+  </si>
+  <si>
+    <t>1|0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relationships |Resent </t>
+  </si>
+  <si>
+    <t>Age|Resent</t>
+  </si>
+  <si>
+    <t>2|0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You know, usually when people complain about detectives 'prying into their personal lives' it isn't quite so literal. Do you have a point you're trying to make, Detective?|*Her knuckles are practically white around the stem of her glass. This ain't exactly your typical 'Shitty ex' response.|Mrs.Scarletta, I'm not implying anything, just a curious girl working a curious job.|Then I suspect you should ask your curious questions elsewhere, Detective.|She spits the last words, turning on her heel. It might not be my case, but there was definitely something going on here. </t>
+  </si>
+  <si>
+    <t>Angry|Angry|Happy|Angry|Sad</t>
+  </si>
+  <si>
+    <t>Angry|Neutral|Angry|Neutral|Neutral|Angry</t>
+  </si>
+  <si>
+    <t>Daria Scarletta|Detective Juels|Daria Scarletta|Detective Juels|Detective Juels|Daria Scarletta</t>
+  </si>
+  <si>
+    <t>3|0|3|0|0|3</t>
   </si>
 </sst>
 </file>
@@ -292,6 +322,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -611,14 +645,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B535539-FE09-464A-9C16-6FD4CB64E674}">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.1796875" style="1" customWidth="1"/>
     <col min="2" max="2" width="36.54296875" style="1" customWidth="1"/>
     <col min="3" max="3" width="43.7265625" style="1" customWidth="1"/>
     <col min="4" max="4" width="13" style="1" customWidth="1"/>
-    <col min="5" max="6" width="11.08984375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.54296875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="11.08984375" style="1" customWidth="1"/>
     <col min="7" max="7" width="11.36328125" style="1" customWidth="1"/>
     <col min="8" max="8" width="17.90625" style="1" customWidth="1"/>
     <col min="9" max="11" width="8.7265625" style="1"/>
@@ -678,34 +713,34 @@
         <v>15</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="G2" s="1">
         <v>0</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="J2" s="1">
         <v>1</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="M2" s="1">
         <v>0</v>
@@ -716,40 +751,40 @@
     </row>
     <row r="3" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="1">
-        <v>0</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="M3" s="1">
         <v>0</v>
@@ -760,40 +795,40 @@
     </row>
     <row r="4" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="C4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="1">
-        <v>0</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="M4" s="1">
         <v>0</v>
@@ -802,42 +837,42 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="116" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G5" s="1">
-        <v>2</v>
+        <v>66</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>70</v>
       </c>
       <c r="H5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="J5" s="1">
         <v>1</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="M5" s="1">
         <v>0</v>
@@ -848,40 +883,40 @@
     </row>
     <row r="6" spans="1:14" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="E6" s="1" t="s">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L6" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
@@ -892,40 +927,40 @@
     </row>
     <row r="7" spans="1:14" ht="145" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="E7" s="1" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G7" s="1">
-        <v>1</v>
+        <v>66</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>67</v>
       </c>
       <c r="H7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="J7" s="1">
         <v>1</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="M7" s="1">
         <v>0</v>
@@ -936,46 +971,90 @@
     </row>
     <row r="8" spans="1:14" ht="87" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="L8" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" s="1">
-        <v>0</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="M8" s="1">
         <v>0</v>
       </c>
       <c r="N8" s="1">
         <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="174" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="J9" s="1">
+        <v>1</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="M9" s="1">
+        <v>0</v>
+      </c>
+      <c r="N9" s="1">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>